<commit_message>
Open Prospecting List tab by default on B2B FL workbook
Moves Prospecting List to first tab position and sets it as the active
sheet so the actual company data shows on open rather than the summary
legend tab.

https://claude.ai/code/session_014Z9j9N5TcCLpqwigG1cFFa
</commit_message>
<xml_diff>
--- a/Magic_B2B_Prospecting_FL_Highlighted.xlsx
+++ b/Magic_B2B_Prospecting_FL_Highlighted.xlsx
@@ -7,8 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="0" xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="23385" tabRatio="0" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="FL Highlights Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Prospecting List" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Prospecting List" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="FL Highlights Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -1264,140 +1264,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="60" customWidth="1" min="1" max="1"/>
-    <col width="100" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="10" t="inlineStr">
-        <is>
-          <t>Florida-Connected B2B Prospects</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="11" t="inlineStr">
-        <is>
-          <t>Legend</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>HQ in FL, dedicated FL business unit/subsidiary, multiple FL offices/branches as a top market, or FL explicitly cited as a strategic market</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="13" t="inlineStr">
-        <is>
-          <t>EDGE</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Some FL operational presence (1-2 offices, regional rep coverage, distribution touch-point) but FL is one of many markets — not dominant</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="11" t="inlineStr">
-        <is>
-          <t>Counts</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>YES — 111 (28 HQ'd in FL + 83 with major FL operations)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>EDGE — 47</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>NO — remaining rows (no meaningful FL connection)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="14" t="inlineStr">
-        <is>
-          <t>Methodology notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="15" t="inlineStr">
-        <is>
-          <t>Pass 1: auto-tagged all 29 companies with HQ listed in Florida (incl. Waste Pro USA — manual correction).</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="15" t="inlineStr">
-        <is>
-          <t>Pass 2: dispatched 6 parallel research agents to assess the remaining ~177 non-FL-HQ companies for major FL operations (multiple FL offices/branches, FL-based subsidiary, FL acquisition history, FL named as top market).</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="15" t="inlineStr">
-        <is>
-          <t>YES = strong evidence FL is a top-tier operational market. EDGE = some FL presence (1-2 offices, regional coverage) but not dominant. NO = no meaningful FL connection beyond standard nationwide footprint.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="15" t="inlineStr">
-        <is>
-          <t>Data corrections: Waste Pro USA HQ is Longwood, FL (source listed 'United States'); Binance YES applies only to Binance.US (Miami) — global Binance.com is a separate entity.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="15" t="inlineStr">
-        <is>
-          <t>For large Fortune 500 companies (JPM, Sysco, GEICO, Spectrum, Toll Brothers), YES required dedicated FL workforce/asset evidence beyond just nationwide operations.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A17:B17"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H207"/>
+  <dimension ref="B2:H207"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11" defaultRowHeight="15.75"/>
   <cols>
     <col width="8.625" customWidth="1" min="1" max="1"/>
@@ -1410,7 +1277,6 @@
     <col width="95" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="16.5" customHeight="1" thickBot="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -7750,4 +7616,137 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>Florida-Connected B2B Prospects</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>Legend</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>HQ in FL, dedicated FL business unit/subsidiary, multiple FL offices/branches as a top market, or FL explicitly cited as a strategic market</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>EDGE</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Some FL operational presence (1-2 offices, regional rep coverage, distribution touch-point) but FL is one of many markets — not dominant</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>Counts</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>YES — 111 (28 HQ'd in FL + 83 with major FL operations)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>EDGE — 47</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>NO — remaining rows (no meaningful FL connection)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>Methodology notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>Pass 1: auto-tagged all 29 companies with HQ listed in Florida (incl. Waste Pro USA — manual correction).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>Pass 2: dispatched 6 parallel research agents to assess the remaining ~177 non-FL-HQ companies for major FL operations (multiple FL offices/branches, FL-based subsidiary, FL acquisition history, FL named as top market).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>YES = strong evidence FL is a top-tier operational market. EDGE = some FL presence (1-2 offices, regional coverage) but not dominant. NO = no meaningful FL connection beyond standard nationwide footprint.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>Data corrections: Waste Pro USA HQ is Longwood, FL (source listed 'United States'); Binance YES applies only to Binance.US (Miami) — global Binance.com is a separate entity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>For large Fortune 500 companies (JPM, Sysco, GEICO, Spectrum, Toll Brothers), YES required dedicated FL workforce/asset evidence beyond just nationwide operations.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A17:B17"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>